<commit_message>
essai python de calcul de ephemerides
</commit_message>
<xml_diff>
--- a/ProjetXLS/PlottingSheet.xlsx
+++ b/ProjetXLS/PlottingSheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\data\git\NavigationBateau\ProjetXLS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpaces\WS\GitHub\Navigation\NavigationBateau\ProjetXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6F5356-3AF4-4728-BBF6-1ADF018BA46F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85CF5C4-059B-4DFC-967F-7BA0F27CD483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sud" sheetId="3" r:id="rId1"/>
@@ -26,6 +26,15 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -43,9 +52,6 @@
     <t>Long</t>
   </si>
   <si>
-    <t>5 Milles</t>
-  </si>
-  <si>
     <t>Sud</t>
   </si>
   <si>
@@ -56,6 +62,9 @@
   </si>
   <si>
     <t>Lat. Nord</t>
+  </si>
+  <si>
+    <t>5 Mn</t>
   </si>
 </sst>
 </file>
@@ -419,24 +428,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
@@ -454,6 +445,24 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -475,7 +484,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2015,7 +2024,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="fr-FR"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -2053,7 +2062,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="499653008"/>
@@ -2145,7 +2154,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="fr-FR"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -2177,7 +2186,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="499652680"/>
@@ -2219,7 +2228,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="fr-FR"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -2233,7 +2242,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3773,7 +3782,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="fr-FR"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -3811,7 +3820,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="499653008"/>
@@ -3903,7 +3912,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="fr-FR"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -3935,7 +3944,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="499652680"/>
@@ -3977,7 +3986,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="fr-FR"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -3991,7 +4000,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -4066,7 +4075,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -5600,7 +5609,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="fr-FR"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -5638,7 +5647,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="499653008"/>
@@ -5730,7 +5739,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="fr-FR"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -5762,7 +5771,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="499652680"/>
@@ -5804,7 +5813,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="fr-FR"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -7838,7 +7847,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:DE111"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.85546875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="2.85546875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="17" width="3.7109375" customWidth="1"/>
     <col min="18" max="18" width="6.28515625" customWidth="1"/>
@@ -7918,28 +7927,28 @@
     </row>
     <row r="2" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S2" s="18"/>
-      <c r="BZ2" s="36" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA2" s="37"/>
+      <c r="BZ2" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="CA2" s="31"/>
       <c r="CB2" s="19"/>
     </row>
     <row r="3" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S3" s="18"/>
-      <c r="BZ3" s="38"/>
-      <c r="CA3" s="39"/>
+      <c r="BZ3" s="32"/>
+      <c r="CA3" s="33"/>
       <c r="CB3" s="19"/>
     </row>
     <row r="4" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S4" s="18"/>
-      <c r="BZ4" s="38"/>
-      <c r="CA4" s="39"/>
+      <c r="BZ4" s="32"/>
+      <c r="CA4" s="33"/>
       <c r="CB4" s="19"/>
     </row>
     <row r="5" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S5" s="18"/>
-      <c r="BZ5" s="40"/>
-      <c r="CA5" s="41"/>
+      <c r="BZ5" s="34"/>
+      <c r="CA5" s="35"/>
       <c r="CB5" s="19"/>
     </row>
     <row r="6" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8090,7 +8099,7 @@
       <c r="S42" s="18"/>
       <c r="CB42" s="19"/>
       <c r="CP42" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:109" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8236,109 +8245,109 @@
       <c r="CB46" s="19"/>
     </row>
     <row r="47" spans="1:109" s="12" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="S47" s="32">
+      <c r="S47" s="38">
         <v>30</v>
       </c>
-      <c r="T47" s="30"/>
-      <c r="X47" s="30">
+      <c r="T47" s="36"/>
+      <c r="X47" s="36">
         <v>25</v>
       </c>
-      <c r="Y47" s="30"/>
-      <c r="AC47" s="30">
+      <c r="Y47" s="36"/>
+      <c r="AC47" s="36">
         <v>20</v>
       </c>
-      <c r="AD47" s="30"/>
-      <c r="AH47" s="30">
+      <c r="AD47" s="36"/>
+      <c r="AH47" s="36">
         <v>15</v>
       </c>
-      <c r="AI47" s="30"/>
-      <c r="AM47" s="30">
+      <c r="AI47" s="36"/>
+      <c r="AM47" s="36">
         <v>10</v>
       </c>
-      <c r="AN47" s="30"/>
-      <c r="AR47" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="AS47" s="30"/>
+      <c r="AN47" s="36"/>
+      <c r="AR47" s="36" t="s">
+        <v>7</v>
+      </c>
+      <c r="AS47" s="36"/>
       <c r="AX47" s="13"/>
-      <c r="BB47" s="30" t="s">
-        <v>5</v>
-      </c>
-      <c r="BC47" s="30"/>
-      <c r="BG47" s="30">
+      <c r="BB47" s="36" t="s">
+        <v>4</v>
+      </c>
+      <c r="BC47" s="36"/>
+      <c r="BG47" s="36">
         <v>50</v>
       </c>
-      <c r="BH47" s="30"/>
-      <c r="BL47" s="30">
+      <c r="BH47" s="36"/>
+      <c r="BL47" s="36">
         <v>45</v>
       </c>
-      <c r="BM47" s="30"/>
-      <c r="BQ47" s="30">
+      <c r="BM47" s="36"/>
+      <c r="BQ47" s="36">
         <v>40</v>
       </c>
-      <c r="BR47" s="30"/>
-      <c r="BV47" s="30">
+      <c r="BR47" s="36"/>
+      <c r="BV47" s="36">
         <v>35</v>
       </c>
-      <c r="BW47" s="30"/>
-      <c r="CA47" s="30">
+      <c r="BW47" s="36"/>
+      <c r="CA47" s="36">
         <v>30</v>
       </c>
-      <c r="CB47" s="31"/>
+      <c r="CB47" s="37"/>
     </row>
     <row r="48" spans="1:109" s="12" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="S48" s="32"/>
-      <c r="T48" s="30"/>
-      <c r="X48" s="30"/>
-      <c r="Y48" s="30"/>
-      <c r="AC48" s="30"/>
-      <c r="AD48" s="30"/>
-      <c r="AH48" s="30"/>
-      <c r="AI48" s="30"/>
-      <c r="AM48" s="30"/>
-      <c r="AN48" s="30"/>
-      <c r="AR48" s="30"/>
-      <c r="AS48" s="30"/>
+      <c r="S48" s="38"/>
+      <c r="T48" s="36"/>
+      <c r="X48" s="36"/>
+      <c r="Y48" s="36"/>
+      <c r="AC48" s="36"/>
+      <c r="AD48" s="36"/>
+      <c r="AH48" s="36"/>
+      <c r="AI48" s="36"/>
+      <c r="AM48" s="36"/>
+      <c r="AN48" s="36"/>
+      <c r="AR48" s="36"/>
+      <c r="AS48" s="36"/>
       <c r="AX48" s="13"/>
-      <c r="BB48" s="30"/>
-      <c r="BC48" s="30"/>
-      <c r="BG48" s="30"/>
-      <c r="BH48" s="30"/>
-      <c r="BL48" s="30"/>
-      <c r="BM48" s="30"/>
-      <c r="BQ48" s="30"/>
-      <c r="BR48" s="30"/>
-      <c r="BV48" s="30"/>
-      <c r="BW48" s="30"/>
-      <c r="CA48" s="30"/>
-      <c r="CB48" s="31"/>
+      <c r="BB48" s="36"/>
+      <c r="BC48" s="36"/>
+      <c r="BG48" s="36"/>
+      <c r="BH48" s="36"/>
+      <c r="BL48" s="36"/>
+      <c r="BM48" s="36"/>
+      <c r="BQ48" s="36"/>
+      <c r="BR48" s="36"/>
+      <c r="BV48" s="36"/>
+      <c r="BW48" s="36"/>
+      <c r="CA48" s="36"/>
+      <c r="CB48" s="37"/>
     </row>
     <row r="49" spans="19:80" s="12" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="S49" s="32"/>
-      <c r="T49" s="30"/>
-      <c r="X49" s="30"/>
-      <c r="Y49" s="30"/>
-      <c r="AC49" s="30"/>
-      <c r="AD49" s="30"/>
-      <c r="AH49" s="30"/>
-      <c r="AI49" s="30"/>
-      <c r="AM49" s="30"/>
-      <c r="AN49" s="30"/>
-      <c r="AR49" s="30"/>
-      <c r="AS49" s="30"/>
+      <c r="S49" s="38"/>
+      <c r="T49" s="36"/>
+      <c r="X49" s="36"/>
+      <c r="Y49" s="36"/>
+      <c r="AC49" s="36"/>
+      <c r="AD49" s="36"/>
+      <c r="AH49" s="36"/>
+      <c r="AI49" s="36"/>
+      <c r="AM49" s="36"/>
+      <c r="AN49" s="36"/>
+      <c r="AR49" s="36"/>
+      <c r="AS49" s="36"/>
       <c r="AX49" s="13"/>
-      <c r="BB49" s="30"/>
-      <c r="BC49" s="30"/>
-      <c r="BG49" s="30"/>
-      <c r="BH49" s="30"/>
-      <c r="BL49" s="30"/>
-      <c r="BM49" s="30"/>
-      <c r="BQ49" s="30"/>
-      <c r="BR49" s="30"/>
-      <c r="BV49" s="30"/>
-      <c r="BW49" s="30"/>
-      <c r="CA49" s="30"/>
-      <c r="CB49" s="31"/>
+      <c r="BB49" s="36"/>
+      <c r="BC49" s="36"/>
+      <c r="BG49" s="36"/>
+      <c r="BH49" s="36"/>
+      <c r="BL49" s="36"/>
+      <c r="BM49" s="36"/>
+      <c r="BQ49" s="36"/>
+      <c r="BR49" s="36"/>
+      <c r="BV49" s="36"/>
+      <c r="BW49" s="36"/>
+      <c r="CA49" s="36"/>
+      <c r="CB49" s="37"/>
     </row>
     <row r="50" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S50" s="18"/>
@@ -9330,6 +9339,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="AR47:AS49"/>
+    <mergeCell ref="S47:T49"/>
+    <mergeCell ref="X47:Y49"/>
+    <mergeCell ref="AC47:AD49"/>
+    <mergeCell ref="AH47:AI49"/>
+    <mergeCell ref="AM47:AN49"/>
     <mergeCell ref="BZ2:CA5"/>
     <mergeCell ref="BB47:BC49"/>
     <mergeCell ref="BG47:BH49"/>
@@ -9337,12 +9352,6 @@
     <mergeCell ref="BQ47:BR49"/>
     <mergeCell ref="BV47:BW49"/>
     <mergeCell ref="CA47:CB49"/>
-    <mergeCell ref="S47:T49"/>
-    <mergeCell ref="X47:Y49"/>
-    <mergeCell ref="AC47:AD49"/>
-    <mergeCell ref="AH47:AI49"/>
-    <mergeCell ref="AM47:AN49"/>
-    <mergeCell ref="AR47:AS49"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -9357,7 +9366,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:DE111"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.85546875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="2.85546875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="17" width="3.7109375" customWidth="1"/>
     <col min="18" max="18" width="6.28515625" customWidth="1"/>
@@ -9437,28 +9446,28 @@
     </row>
     <row r="2" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S2" s="18"/>
-      <c r="BZ2" s="36" t="s">
-        <v>7</v>
-      </c>
-      <c r="CA2" s="37"/>
+      <c r="BZ2" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA2" s="31"/>
       <c r="CB2" s="19"/>
     </row>
     <row r="3" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S3" s="18"/>
-      <c r="BZ3" s="38"/>
-      <c r="CA3" s="39"/>
+      <c r="BZ3" s="32"/>
+      <c r="CA3" s="33"/>
       <c r="CB3" s="19"/>
     </row>
     <row r="4" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S4" s="18"/>
-      <c r="BZ4" s="38"/>
-      <c r="CA4" s="39"/>
+      <c r="BZ4" s="32"/>
+      <c r="CA4" s="33"/>
       <c r="CB4" s="19"/>
     </row>
     <row r="5" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S5" s="18"/>
-      <c r="BZ5" s="40"/>
-      <c r="CA5" s="41"/>
+      <c r="BZ5" s="34"/>
+      <c r="CA5" s="35"/>
       <c r="CB5" s="19"/>
     </row>
     <row r="6" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9752,109 +9761,109 @@
       <c r="CB46" s="19"/>
     </row>
     <row r="47" spans="1:109" s="12" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="S47" s="32">
+      <c r="S47" s="38">
         <v>30</v>
       </c>
-      <c r="T47" s="30"/>
-      <c r="X47" s="30">
+      <c r="T47" s="36"/>
+      <c r="X47" s="36">
         <v>35</v>
       </c>
-      <c r="Y47" s="30"/>
-      <c r="AC47" s="30">
+      <c r="Y47" s="36"/>
+      <c r="AC47" s="36">
         <v>40</v>
       </c>
-      <c r="AD47" s="30"/>
-      <c r="AH47" s="30">
+      <c r="AD47" s="36"/>
+      <c r="AH47" s="36">
         <v>45</v>
       </c>
-      <c r="AI47" s="30"/>
-      <c r="AM47" s="30">
+      <c r="AI47" s="36"/>
+      <c r="AM47" s="36">
         <v>50</v>
       </c>
-      <c r="AN47" s="30"/>
-      <c r="AR47" s="30">
+      <c r="AN47" s="36"/>
+      <c r="AR47" s="36">
         <v>55</v>
       </c>
-      <c r="AS47" s="30"/>
+      <c r="AS47" s="36"/>
       <c r="AX47" s="13"/>
-      <c r="BB47" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="BC47" s="30"/>
-      <c r="BG47" s="30">
+      <c r="BB47" s="36" t="s">
+        <v>7</v>
+      </c>
+      <c r="BC47" s="36"/>
+      <c r="BG47" s="36">
         <v>10</v>
       </c>
-      <c r="BH47" s="30"/>
-      <c r="BL47" s="30">
+      <c r="BH47" s="36"/>
+      <c r="BL47" s="36">
         <v>15</v>
       </c>
-      <c r="BM47" s="30"/>
-      <c r="BQ47" s="30">
+      <c r="BM47" s="36"/>
+      <c r="BQ47" s="36">
         <v>20</v>
       </c>
-      <c r="BR47" s="30"/>
-      <c r="BV47" s="30">
+      <c r="BR47" s="36"/>
+      <c r="BV47" s="36">
         <v>25</v>
       </c>
-      <c r="BW47" s="30"/>
-      <c r="CA47" s="30">
+      <c r="BW47" s="36"/>
+      <c r="CA47" s="36">
         <v>30</v>
       </c>
-      <c r="CB47" s="31"/>
+      <c r="CB47" s="37"/>
     </row>
     <row r="48" spans="1:109" s="12" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="S48" s="32"/>
-      <c r="T48" s="30"/>
-      <c r="X48" s="30"/>
-      <c r="Y48" s="30"/>
-      <c r="AC48" s="30"/>
-      <c r="AD48" s="30"/>
-      <c r="AH48" s="30"/>
-      <c r="AI48" s="30"/>
-      <c r="AM48" s="30"/>
-      <c r="AN48" s="30"/>
-      <c r="AR48" s="30"/>
-      <c r="AS48" s="30"/>
+      <c r="S48" s="38"/>
+      <c r="T48" s="36"/>
+      <c r="X48" s="36"/>
+      <c r="Y48" s="36"/>
+      <c r="AC48" s="36"/>
+      <c r="AD48" s="36"/>
+      <c r="AH48" s="36"/>
+      <c r="AI48" s="36"/>
+      <c r="AM48" s="36"/>
+      <c r="AN48" s="36"/>
+      <c r="AR48" s="36"/>
+      <c r="AS48" s="36"/>
       <c r="AX48" s="13"/>
-      <c r="BB48" s="30"/>
-      <c r="BC48" s="30"/>
-      <c r="BG48" s="30"/>
-      <c r="BH48" s="30"/>
-      <c r="BL48" s="30"/>
-      <c r="BM48" s="30"/>
-      <c r="BQ48" s="30"/>
-      <c r="BR48" s="30"/>
-      <c r="BV48" s="30"/>
-      <c r="BW48" s="30"/>
-      <c r="CA48" s="30"/>
-      <c r="CB48" s="31"/>
+      <c r="BB48" s="36"/>
+      <c r="BC48" s="36"/>
+      <c r="BG48" s="36"/>
+      <c r="BH48" s="36"/>
+      <c r="BL48" s="36"/>
+      <c r="BM48" s="36"/>
+      <c r="BQ48" s="36"/>
+      <c r="BR48" s="36"/>
+      <c r="BV48" s="36"/>
+      <c r="BW48" s="36"/>
+      <c r="CA48" s="36"/>
+      <c r="CB48" s="37"/>
     </row>
     <row r="49" spans="19:80" s="12" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="S49" s="32"/>
-      <c r="T49" s="30"/>
-      <c r="X49" s="30"/>
-      <c r="Y49" s="30"/>
-      <c r="AC49" s="30"/>
-      <c r="AD49" s="30"/>
-      <c r="AH49" s="30"/>
-      <c r="AI49" s="30"/>
-      <c r="AM49" s="30"/>
-      <c r="AN49" s="30"/>
-      <c r="AR49" s="30"/>
-      <c r="AS49" s="30"/>
+      <c r="S49" s="38"/>
+      <c r="T49" s="36"/>
+      <c r="X49" s="36"/>
+      <c r="Y49" s="36"/>
+      <c r="AC49" s="36"/>
+      <c r="AD49" s="36"/>
+      <c r="AH49" s="36"/>
+      <c r="AI49" s="36"/>
+      <c r="AM49" s="36"/>
+      <c r="AN49" s="36"/>
+      <c r="AR49" s="36"/>
+      <c r="AS49" s="36"/>
       <c r="AX49" s="13"/>
-      <c r="BB49" s="30"/>
-      <c r="BC49" s="30"/>
-      <c r="BG49" s="30"/>
-      <c r="BH49" s="30"/>
-      <c r="BL49" s="30"/>
-      <c r="BM49" s="30"/>
-      <c r="BQ49" s="30"/>
-      <c r="BR49" s="30"/>
-      <c r="BV49" s="30"/>
-      <c r="BW49" s="30"/>
-      <c r="CA49" s="30"/>
-      <c r="CB49" s="31"/>
+      <c r="BB49" s="36"/>
+      <c r="BC49" s="36"/>
+      <c r="BG49" s="36"/>
+      <c r="BH49" s="36"/>
+      <c r="BL49" s="36"/>
+      <c r="BM49" s="36"/>
+      <c r="BQ49" s="36"/>
+      <c r="BR49" s="36"/>
+      <c r="BV49" s="36"/>
+      <c r="BW49" s="36"/>
+      <c r="CA49" s="36"/>
+      <c r="CB49" s="37"/>
     </row>
     <row r="50" spans="19:80" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="S50" s="18"/>
@@ -10873,7 +10882,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:DR62"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="2.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="43" max="43" width="0.85546875" style="8" customWidth="1"/>
     <col min="44" max="44" width="1" customWidth="1"/>
@@ -10930,11 +10939,11 @@
       <c r="AQ1" s="6"/>
       <c r="AR1" s="2"/>
       <c r="AS1" s="3"/>
-      <c r="AT1" s="34">
+      <c r="AT1" s="41">
         <v>30</v>
       </c>
-      <c r="AU1" s="34"/>
-      <c r="AV1" s="34"/>
+      <c r="AU1" s="41"/>
+      <c r="AV1" s="41"/>
       <c r="AW1" s="3"/>
       <c r="AX1" s="3"/>
       <c r="AY1" s="3"/>
@@ -10985,9 +10994,9 @@
       <c r="AQ2" s="5"/>
       <c r="AR2" s="4"/>
       <c r="AS2" s="4"/>
-      <c r="AT2" s="33"/>
-      <c r="AU2" s="33"/>
-      <c r="AV2" s="33"/>
+      <c r="AT2" s="39"/>
+      <c r="AU2" s="39"/>
+      <c r="AV2" s="39"/>
       <c r="CN2" s="10"/>
     </row>
     <row r="3" spans="1:92" x14ac:dyDescent="0.25">
@@ -11010,11 +11019,11 @@
       <c r="AQ6" s="5"/>
       <c r="AR6" s="1"/>
       <c r="AS6" s="4"/>
-      <c r="AT6" s="33">
+      <c r="AT6" s="39">
         <v>25</v>
       </c>
-      <c r="AU6" s="33"/>
-      <c r="AV6" s="33"/>
+      <c r="AU6" s="39"/>
+      <c r="AV6" s="39"/>
       <c r="CN6" s="10"/>
     </row>
     <row r="7" spans="1:92" x14ac:dyDescent="0.25">
@@ -11022,9 +11031,9 @@
       <c r="AQ7" s="5"/>
       <c r="AR7" s="4"/>
       <c r="AS7" s="4"/>
-      <c r="AT7" s="33"/>
-      <c r="AU7" s="33"/>
-      <c r="AV7" s="33"/>
+      <c r="AT7" s="39"/>
+      <c r="AU7" s="39"/>
+      <c r="AV7" s="39"/>
       <c r="CN7" s="10"/>
     </row>
     <row r="8" spans="1:92" x14ac:dyDescent="0.25">
@@ -11047,11 +11056,11 @@
       <c r="AQ11" s="5"/>
       <c r="AR11" s="1"/>
       <c r="AS11" s="4"/>
-      <c r="AT11" s="33">
+      <c r="AT11" s="39">
         <v>20</v>
       </c>
-      <c r="AU11" s="33"/>
-      <c r="AV11" s="33"/>
+      <c r="AU11" s="39"/>
+      <c r="AV11" s="39"/>
       <c r="CN11" s="10"/>
     </row>
     <row r="12" spans="1:92" x14ac:dyDescent="0.25">
@@ -11059,9 +11068,9 @@
       <c r="AQ12" s="5"/>
       <c r="AR12" s="4"/>
       <c r="AS12" s="4"/>
-      <c r="AT12" s="33"/>
-      <c r="AU12" s="33"/>
-      <c r="AV12" s="33"/>
+      <c r="AT12" s="39"/>
+      <c r="AU12" s="39"/>
+      <c r="AV12" s="39"/>
       <c r="CN12" s="10"/>
     </row>
     <row r="13" spans="1:92" x14ac:dyDescent="0.25">
@@ -11083,20 +11092,20 @@
       <c r="A16" s="8"/>
       <c r="AQ16" s="6"/>
       <c r="AR16" s="1"/>
-      <c r="AT16" s="33">
+      <c r="AT16" s="39">
         <v>15</v>
       </c>
-      <c r="AU16" s="33"/>
-      <c r="AV16" s="33"/>
+      <c r="AU16" s="39"/>
+      <c r="AV16" s="39"/>
       <c r="CN16" s="10"/>
     </row>
     <row r="17" spans="1:92" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
       <c r="AQ17" s="5"/>
       <c r="AR17" s="4"/>
-      <c r="AT17" s="33"/>
-      <c r="AU17" s="33"/>
-      <c r="AV17" s="33"/>
+      <c r="AT17" s="39"/>
+      <c r="AU17" s="39"/>
+      <c r="AV17" s="39"/>
       <c r="CN17" s="10"/>
     </row>
     <row r="18" spans="1:92" x14ac:dyDescent="0.25">
@@ -11119,11 +11128,11 @@
       <c r="AQ21" s="5"/>
       <c r="AR21" s="1"/>
       <c r="AS21" s="4"/>
-      <c r="AT21" s="33">
+      <c r="AT21" s="39">
         <v>10</v>
       </c>
-      <c r="AU21" s="33"/>
-      <c r="AV21" s="33"/>
+      <c r="AU21" s="39"/>
+      <c r="AV21" s="39"/>
       <c r="CN21" s="10"/>
     </row>
     <row r="22" spans="1:92" x14ac:dyDescent="0.25">
@@ -11131,9 +11140,9 @@
       <c r="AQ22" s="5"/>
       <c r="AR22" s="4"/>
       <c r="AS22" s="4"/>
-      <c r="AT22" s="33"/>
-      <c r="AU22" s="33"/>
-      <c r="AV22" s="33"/>
+      <c r="AT22" s="39"/>
+      <c r="AU22" s="39"/>
+      <c r="AV22" s="39"/>
       <c r="CN22" s="10"/>
     </row>
     <row r="23" spans="1:92" x14ac:dyDescent="0.25">
@@ -11156,11 +11165,11 @@
       <c r="AQ26" s="5"/>
       <c r="AR26" s="1"/>
       <c r="AS26" s="4"/>
-      <c r="AT26" s="33" t="s">
+      <c r="AT26" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="AU26" s="33"/>
-      <c r="AV26" s="33"/>
+      <c r="AU26" s="39"/>
+      <c r="AV26" s="39"/>
       <c r="CN26" s="10"/>
     </row>
     <row r="27" spans="1:92" x14ac:dyDescent="0.25">
@@ -11168,9 +11177,9 @@
       <c r="AQ27" s="5"/>
       <c r="AR27" s="4"/>
       <c r="AS27" s="4"/>
-      <c r="AT27" s="33"/>
-      <c r="AU27" s="33"/>
-      <c r="AV27" s="33"/>
+      <c r="AT27" s="39"/>
+      <c r="AU27" s="39"/>
+      <c r="AV27" s="39"/>
       <c r="CN27" s="10"/>
     </row>
     <row r="28" spans="1:92" x14ac:dyDescent="0.25">
@@ -11224,11 +11233,11 @@
       <c r="AQ36" s="5"/>
       <c r="AR36" s="1"/>
       <c r="AS36" s="4"/>
-      <c r="AT36" s="33">
+      <c r="AT36" s="39">
         <v>55</v>
       </c>
-      <c r="AU36" s="33"/>
-      <c r="AV36" s="33"/>
+      <c r="AU36" s="39"/>
+      <c r="AV36" s="39"/>
       <c r="CN36" s="10"/>
     </row>
     <row r="37" spans="1:122" x14ac:dyDescent="0.25">
@@ -11236,9 +11245,9 @@
       <c r="AQ37" s="5"/>
       <c r="AR37" s="4"/>
       <c r="AS37" s="4"/>
-      <c r="AT37" s="33"/>
-      <c r="AU37" s="33"/>
-      <c r="AV37" s="33"/>
+      <c r="AT37" s="39"/>
+      <c r="AU37" s="39"/>
+      <c r="AV37" s="39"/>
       <c r="CN37" s="10"/>
     </row>
     <row r="38" spans="1:122" x14ac:dyDescent="0.25">
@@ -11261,11 +11270,11 @@
       <c r="AQ41" s="5"/>
       <c r="AR41" s="1"/>
       <c r="AS41" s="4"/>
-      <c r="AT41" s="33">
+      <c r="AT41" s="39">
         <v>50</v>
       </c>
-      <c r="AU41" s="33"/>
-      <c r="AV41" s="33"/>
+      <c r="AU41" s="39"/>
+      <c r="AV41" s="39"/>
       <c r="CN41" s="10"/>
     </row>
     <row r="42" spans="1:122" x14ac:dyDescent="0.25">
@@ -11273,9 +11282,9 @@
       <c r="AQ42" s="5"/>
       <c r="AR42" s="4"/>
       <c r="AS42" s="4"/>
-      <c r="AT42" s="33"/>
-      <c r="AU42" s="33"/>
-      <c r="AV42" s="33"/>
+      <c r="AT42" s="39"/>
+      <c r="AU42" s="39"/>
+      <c r="AV42" s="39"/>
       <c r="CN42" s="10"/>
     </row>
     <row r="43" spans="1:122" x14ac:dyDescent="0.25">
@@ -11297,11 +11306,11 @@
       <c r="A46" s="8"/>
       <c r="AQ46" s="6"/>
       <c r="AR46" s="1"/>
-      <c r="AT46" s="33">
+      <c r="AT46" s="39">
         <v>45</v>
       </c>
-      <c r="AU46" s="33"/>
-      <c r="AV46" s="33"/>
+      <c r="AU46" s="39"/>
+      <c r="AV46" s="39"/>
       <c r="CN46" s="10"/>
       <c r="CY46" t="s">
         <v>1</v>
@@ -11386,9 +11395,9 @@
       <c r="A47" s="8"/>
       <c r="AQ47" s="5"/>
       <c r="AR47" s="4"/>
-      <c r="AT47" s="33"/>
-      <c r="AU47" s="33"/>
-      <c r="AV47" s="33"/>
+      <c r="AT47" s="39"/>
+      <c r="AU47" s="39"/>
+      <c r="AV47" s="39"/>
       <c r="CN47" s="10"/>
       <c r="CY47" t="s">
         <v>2</v>
@@ -11727,11 +11736,11 @@
       <c r="AQ51" s="5"/>
       <c r="AR51" s="1"/>
       <c r="AS51" s="4"/>
-      <c r="AT51" s="33">
+      <c r="AT51" s="39">
         <v>40</v>
       </c>
-      <c r="AU51" s="33"/>
-      <c r="AV51" s="33"/>
+      <c r="AU51" s="39"/>
+      <c r="AV51" s="39"/>
       <c r="CN51" s="10"/>
       <c r="CY51" t="s">
         <v>2</v>
@@ -11818,9 +11827,9 @@
       <c r="AQ52" s="5"/>
       <c r="AR52" s="4"/>
       <c r="AS52" s="4"/>
-      <c r="AT52" s="33"/>
-      <c r="AU52" s="33"/>
-      <c r="AV52" s="33"/>
+      <c r="AT52" s="39"/>
+      <c r="AU52" s="39"/>
+      <c r="AV52" s="39"/>
       <c r="CN52" s="10"/>
       <c r="CY52" t="s">
         <v>2</v>
@@ -12080,11 +12089,11 @@
       <c r="AQ56" s="5"/>
       <c r="AR56" s="1"/>
       <c r="AS56" s="4"/>
-      <c r="AT56" s="33">
+      <c r="AT56" s="39">
         <v>35</v>
       </c>
-      <c r="AU56" s="33"/>
-      <c r="AV56" s="33"/>
+      <c r="AU56" s="39"/>
+      <c r="AV56" s="39"/>
       <c r="CN56" s="10"/>
     </row>
     <row r="57" spans="1:122" x14ac:dyDescent="0.25">
@@ -12092,9 +12101,9 @@
       <c r="AQ57" s="5"/>
       <c r="AR57" s="4"/>
       <c r="AS57" s="4"/>
-      <c r="AT57" s="33"/>
-      <c r="AU57" s="33"/>
-      <c r="AV57" s="33"/>
+      <c r="AT57" s="39"/>
+      <c r="AU57" s="39"/>
+      <c r="AV57" s="39"/>
       <c r="CN57" s="10"/>
     </row>
     <row r="58" spans="1:122" x14ac:dyDescent="0.25">
@@ -12116,11 +12125,11 @@
       <c r="A61" s="8"/>
       <c r="AQ61" s="6"/>
       <c r="AR61" s="1"/>
-      <c r="AT61" s="33">
+      <c r="AT61" s="39">
         <v>30</v>
       </c>
-      <c r="AU61" s="33"/>
-      <c r="AV61" s="33"/>
+      <c r="AU61" s="39"/>
+      <c r="AV61" s="39"/>
       <c r="CN61" s="10"/>
     </row>
     <row r="62" spans="1:122" x14ac:dyDescent="0.25">
@@ -12169,9 +12178,9 @@
       <c r="AQ62" s="5"/>
       <c r="AR62" s="1"/>
       <c r="AS62" s="1"/>
-      <c r="AT62" s="35"/>
-      <c r="AU62" s="35"/>
-      <c r="AV62" s="35"/>
+      <c r="AT62" s="40"/>
+      <c r="AU62" s="40"/>
+      <c r="AV62" s="40"/>
       <c r="AW62" s="1"/>
       <c r="AX62" s="1"/>
       <c r="AY62" s="1"/>
@@ -12219,18 +12228,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AT26:AV27"/>
+    <mergeCell ref="AT1:AV2"/>
+    <mergeCell ref="AT6:AV7"/>
+    <mergeCell ref="AT11:AV12"/>
+    <mergeCell ref="AT16:AV17"/>
+    <mergeCell ref="AT21:AV22"/>
     <mergeCell ref="AT56:AV57"/>
     <mergeCell ref="AT61:AV62"/>
     <mergeCell ref="AT36:AV37"/>
     <mergeCell ref="AT41:AV42"/>
     <mergeCell ref="AT46:AV47"/>
     <mergeCell ref="AT51:AV52"/>
-    <mergeCell ref="AT26:AV27"/>
-    <mergeCell ref="AT1:AV2"/>
-    <mergeCell ref="AT6:AV7"/>
-    <mergeCell ref="AT11:AV12"/>
-    <mergeCell ref="AT16:AV17"/>
-    <mergeCell ref="AT21:AV22"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>